<commit_message>
updated timeClips. minor updates.
</commit_message>
<xml_diff>
--- a/timeClips_perSite.xlsx
+++ b/timeClips_perSite.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cawater.sharepoint.com/sites/dwr-frpa/Water Quality Lab/Data Processing/R Files/Processing_SondeData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="445" documentId="8_{EF64B285-CCF4-424B-BA3C-1748E9659AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2DB83B5-131E-4C57-9833-B7DCC23B9B39}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="8_{EF64B285-CCF4-424B-BA3C-1748E9659AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CF78E24-CCB7-43F6-A039-24E478D6E705}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="6" xr2:uid="{A7710E3F-3C9F-4B8D-9D0A-1617AFBC969D}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A7710E3F-3C9F-4B8D-9D0A-1617AFBC969D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Arnold" sheetId="1" r:id="rId1"/>
-    <sheet name="Arnold-Ext" sheetId="2" r:id="rId2"/>
-    <sheet name="Bradmoor" sheetId="3" r:id="rId3"/>
-    <sheet name="Bradmoor-Ext" sheetId="4" r:id="rId4"/>
+    <sheet name="ARN" sheetId="1" r:id="rId1"/>
+    <sheet name="ARN-Ext" sheetId="2" r:id="rId2"/>
+    <sheet name="BRD" sheetId="3" r:id="rId3"/>
+    <sheet name="BRD-Ext" sheetId="4" r:id="rId4"/>
     <sheet name="DKR" sheetId="16" r:id="rId5"/>
     <sheet name="DKR-old" sheetId="12" r:id="rId6"/>
     <sheet name="LOS" sheetId="6" r:id="rId7"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="54">
   <si>
     <t>Site</t>
   </si>
@@ -1483,7 +1483,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{720C55ED-DAB0-40F3-AA24-B9DA7F41F83F}">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="10.140625" bestFit="1" customWidth="1"/>
@@ -1491,7 +1491,7 @@
     <col min="8" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1531,7 +1531,7 @@
         <v>1515</v>
       </c>
       <c r="D2" s="7">
-        <f t="shared" ref="D2:D47" si="0">TIME(LEFT(C2,LEN(C2)-2),RIGHT(C2,2),0)</f>
+        <f t="shared" ref="D2:D46" si="0">TIME(LEFT(C2,LEN(C2)-2),RIGHT(C2,2),0)</f>
         <v>0.63541666666666663</v>
       </c>
       <c r="E2" s="1">
@@ -1541,19 +1541,19 @@
         <v>1315</v>
       </c>
       <c r="G2" s="7">
-        <f t="shared" ref="G2:G47" si="1">TIME(LEFT(F2,LEN(F2)-2),RIGHT(F2,2),0)</f>
+        <f t="shared" ref="G2:G46" si="1">TIME(LEFT(F2,LEN(F2)-2),RIGHT(F2,2),0)</f>
         <v>0.55208333333333337</v>
       </c>
       <c r="H2" s="8">
-        <f t="shared" ref="H2:H47" si="2">B2+D2</f>
+        <f t="shared" ref="H2:H46" si="2">B2+D2</f>
         <v>44655.635416666664</v>
       </c>
       <c r="I2" s="8">
-        <f t="shared" ref="I2:I47" si="3">E2+G2</f>
+        <f t="shared" ref="I2:I46" si="3">E2+G2</f>
         <v>44693.552083333336</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -1586,7 +1586,7 @@
         <v>44735.5625</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>44</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>44782.479166666664</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>44826.427083333336</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>44852.427083333336</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>44887.46875</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -1751,40 +1751,40 @@
         <v>44924.427083333336</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>44</v>
       </c>
       <c r="B9" s="1">
         <v>44924</v>
       </c>
-      <c r="C9" s="9">
-        <v>0.48853009259259261</v>
+      <c r="C9">
+        <v>1143</v>
       </c>
       <c r="D9" s="7">
         <f t="shared" si="0"/>
-        <v>6.458333333333334E-2</v>
+        <v>0.48819444444444443</v>
       </c>
       <c r="E9" s="1">
         <v>44964</v>
       </c>
-      <c r="F9" s="9">
-        <v>0.44686342592592593</v>
+      <c r="F9">
+        <v>1043</v>
       </c>
       <c r="G9" s="7">
         <f t="shared" si="1"/>
-        <v>1.8055555555555554E-2</v>
+        <v>0.4465277777777778</v>
       </c>
       <c r="H9" s="8">
         <f t="shared" si="2"/>
-        <v>44924.064583333333</v>
+        <v>44924.488194444442</v>
       </c>
       <c r="I9" s="8">
         <f t="shared" si="3"/>
-        <v>44964.018055555556</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>44964.446527777778</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>44</v>
       </c>
@@ -1816,8 +1816,9 @@
         <f t="shared" si="3"/>
         <v>45001.552083333336</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -1850,7 +1851,7 @@
         <v>45041.427083333336</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1882,8 +1883,9 @@
         <f t="shared" si="3"/>
         <v>45078.46875</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L12" s="9"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -1916,7 +1918,7 @@
         <v>45118.447916666664</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -1949,7 +1951,7 @@
         <v>45152.510416666664</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>44</v>
       </c>
@@ -1982,7 +1984,7 @@
         <v>45194.4375</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -3003,33 +3005,6 @@
       <c r="I46" s="8">
         <f t="shared" si="3"/>
         <v>46127.427083333336</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>44</v>
-      </c>
-      <c r="B47" s="1">
-        <v>46127</v>
-      </c>
-      <c r="C47">
-        <v>1130</v>
-      </c>
-      <c r="D47" s="7">
-        <f t="shared" si="0"/>
-        <v>0.47916666666666669</v>
-      </c>
-      <c r="G47" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H47" s="8">
-        <f t="shared" si="2"/>
-        <v>46127.479166666664</v>
-      </c>
-      <c r="I47" s="8" t="e">
-        <f t="shared" si="3"/>
-        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -4238,7 +4213,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A78C30C8-7943-4EDB-92A8-475AC6341F00}">
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
@@ -4286,7 +4261,7 @@
         <v>1100</v>
       </c>
       <c r="D2" s="7">
-        <f t="shared" ref="D2:D36" si="0">TIME(LEFT(C2,LEN(C2)-2),RIGHT(C2,2),0)</f>
+        <f t="shared" ref="D2:D35" si="0">TIME(LEFT(C2,LEN(C2)-2),RIGHT(C2,2),0)</f>
         <v>0.45833333333333331</v>
       </c>
       <c r="E2" s="1">
@@ -4296,15 +4271,15 @@
         <v>1230</v>
       </c>
       <c r="G2" s="7">
-        <f t="shared" ref="G2:G36" si="1">TIME(LEFT(F2,LEN(F2)-2),RIGHT(F2,2),0)</f>
+        <f t="shared" ref="G2:G35" si="1">TIME(LEFT(F2,LEN(F2)-2),RIGHT(F2,2),0)</f>
         <v>0.52083333333333337</v>
       </c>
       <c r="H2" s="8">
-        <f t="shared" ref="H2:H36" si="2">B2+D2</f>
+        <f t="shared" ref="H2:H35" si="2">B2+D2</f>
         <v>44952.458333333336</v>
       </c>
       <c r="I2" s="8">
-        <f t="shared" ref="I2:I36" si="3">E2+G2</f>
+        <f t="shared" ref="I2:I35" si="3">E2+G2</f>
         <v>44994.520833333336</v>
       </c>
     </row>
@@ -5395,33 +5370,6 @@
       <c r="I35" s="8">
         <f t="shared" si="3"/>
         <v>46107.375</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>47</v>
-      </c>
-      <c r="B36" s="1">
-        <v>46107</v>
-      </c>
-      <c r="C36">
-        <v>1015</v>
-      </c>
-      <c r="D36" s="7">
-        <f t="shared" si="0"/>
-        <v>0.42708333333333331</v>
-      </c>
-      <c r="G36" s="7" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H36" s="8">
-        <f t="shared" si="2"/>
-        <v>46107.427083333336</v>
-      </c>
-      <c r="I36" s="8" t="e">
-        <f t="shared" si="3"/>
-        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>